<commit_message>
feat: evolve universal bank BCTC schema
</commit_message>
<xml_diff>
--- a/template/Bank_LCTT_ReportNormId.v2.xlsx
+++ b/template/Bank_LCTT_ReportNormId.v2.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="75">
   <si>
     <t>ReportNormId</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t>Tiền thu/(chi) đầu tư, góp vốn vào các đơn vị khác</t>
+  </si>
+  <si>
+    <t>Tiền thu/(chi) bất động sản đầu tư</t>
   </si>
 </sst>
 </file>
@@ -593,7 +596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1577,10 +1580,10 @@
         <v>88</v>
       </c>
       <c r="B90">
-        <v>4144</v>
+        <v>6034</v>
       </c>
       <c r="C90" t="s">
-        <v>40</v>
+        <v>74</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -1588,10 +1591,10 @@
         <v>89</v>
       </c>
       <c r="B91">
-        <v>4145</v>
+        <v>4144</v>
       </c>
       <c r="C91" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -1599,10 +1602,10 @@
         <v>90</v>
       </c>
       <c r="B92">
-        <v>4146</v>
+        <v>4145</v>
       </c>
       <c r="C92" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -1610,10 +1613,10 @@
         <v>91</v>
       </c>
       <c r="B93">
-        <v>5714</v>
+        <v>4146</v>
       </c>
       <c r="C93" t="s">
-        <v>73</v>
+        <v>42</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -1621,10 +1624,10 @@
         <v>92</v>
       </c>
       <c r="B94">
-        <v>4120</v>
+        <v>5714</v>
       </c>
       <c r="C94" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -1632,10 +1635,10 @@
         <v>93</v>
       </c>
       <c r="B95">
-        <v>4121</v>
+        <v>4120</v>
       </c>
       <c r="C95" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -1643,10 +1646,10 @@
         <v>94</v>
       </c>
       <c r="B96">
-        <v>4147</v>
+        <v>4121</v>
       </c>
       <c r="C96" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -1654,10 +1657,10 @@
         <v>95</v>
       </c>
       <c r="B97">
-        <v>4111</v>
+        <v>4147</v>
       </c>
       <c r="C97" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -1665,10 +1668,10 @@
         <v>96</v>
       </c>
       <c r="B98">
-        <v>4106</v>
+        <v>4111</v>
       </c>
       <c r="C98" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -1676,10 +1679,10 @@
         <v>97</v>
       </c>
       <c r="B99">
-        <v>4148</v>
+        <v>4106</v>
       </c>
       <c r="C99" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -1687,10 +1690,10 @@
         <v>98</v>
       </c>
       <c r="B100">
-        <v>4149</v>
+        <v>4148</v>
       </c>
       <c r="C100" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -1698,10 +1701,10 @@
         <v>99</v>
       </c>
       <c r="B101">
-        <v>4150</v>
+        <v>4149</v>
       </c>
       <c r="C101" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -1709,10 +1712,10 @@
         <v>100</v>
       </c>
       <c r="B102">
-        <v>4153</v>
+        <v>4150</v>
       </c>
       <c r="C102" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -1720,10 +1723,10 @@
         <v>101</v>
       </c>
       <c r="B103">
-        <v>4151</v>
+        <v>4153</v>
       </c>
       <c r="C103" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -1731,10 +1734,10 @@
         <v>102</v>
       </c>
       <c r="B104">
-        <v>4152</v>
+        <v>4151</v>
       </c>
       <c r="C104" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -1742,10 +1745,10 @@
         <v>103</v>
       </c>
       <c r="B105">
-        <v>4112</v>
+        <v>4152</v>
       </c>
       <c r="C105" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -1753,10 +1756,10 @@
         <v>104</v>
       </c>
       <c r="B106">
-        <v>4114</v>
+        <v>4112</v>
       </c>
       <c r="C106" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -1764,10 +1767,10 @@
         <v>105</v>
       </c>
       <c r="B107">
-        <v>4115</v>
+        <v>4114</v>
       </c>
       <c r="C107" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -1775,10 +1778,10 @@
         <v>106</v>
       </c>
       <c r="B108">
-        <v>4117</v>
+        <v>4115</v>
       </c>
       <c r="C108" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -1786,9 +1789,20 @@
         <v>107</v>
       </c>
       <c r="B109">
+        <v>4117</v>
+      </c>
+      <c r="C109" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3">
+      <c r="A110" s="1">
+        <v>108</v>
+      </c>
+      <c r="B110">
         <v>4116</v>
       </c>
-      <c r="C109" t="s">
+      <c r="C110" t="s">
         <v>58</v>
       </c>
     </row>

</xml_diff>